<commit_message>
Corrected typo (podpis - Małachowski)
</commit_message>
<xml_diff>
--- a/data/opis_uzupelniony.xlsx
+++ b/data/opis_uzupelniony.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="784" uniqueCount="254">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="784" uniqueCount="253">
   <si>
     <t xml:space="preserve">NAZWA</t>
   </si>
@@ -527,9 +527,6 @@
   </si>
   <si>
     <t xml:space="preserve">ASC20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">podpis -Małachowski</t>
   </si>
   <si>
     <t xml:space="preserve">ASC20A</t>
@@ -791,7 +788,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -827,12 +824,6 @@
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="0"/>
     </font>
   </fonts>
   <fills count="2">
@@ -877,7 +868,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -895,10 +886,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1857,7 +1844,7 @@
       <c r="B55" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="C55" s="5" t="s">
+      <c r="C55" s="2" t="s">
         <v>5</v>
       </c>
       <c r="D55" s="2"/>
@@ -1869,7 +1856,7 @@
       <c r="B56" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="C56" s="5" t="s">
+      <c r="C56" s="2" t="s">
         <v>5</v>
       </c>
       <c r="D56" s="2"/>
@@ -1881,7 +1868,7 @@
       <c r="B57" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="C57" s="5" t="s">
+      <c r="C57" s="2" t="s">
         <v>5</v>
       </c>
       <c r="D57" s="2"/>
@@ -1893,7 +1880,7 @@
       <c r="B58" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="C58" s="5" t="s">
+      <c r="C58" s="2" t="s">
         <v>5</v>
       </c>
       <c r="D58" s="2"/>
@@ -1905,7 +1892,7 @@
       <c r="B59" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="C59" s="5" t="s">
+      <c r="C59" s="2" t="s">
         <v>5</v>
       </c>
       <c r="D59" s="2"/>
@@ -1917,7 +1904,7 @@
       <c r="B60" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="C60" s="5" t="s">
+      <c r="C60" s="2" t="s">
         <v>5</v>
       </c>
       <c r="D60" s="2"/>
@@ -3028,12 +3015,12 @@
         <v>156</v>
       </c>
       <c r="E139" s="2" t="s">
-        <v>169</v>
+        <v>6</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B140" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C140" s="2" t="s">
         <v>83</v>
@@ -3042,12 +3029,12 @@
         <v>156</v>
       </c>
       <c r="E140" s="2" t="s">
-        <v>169</v>
+        <v>6</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B141" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C141" s="2" t="s">
         <v>83</v>
@@ -3056,12 +3043,12 @@
         <v>156</v>
       </c>
       <c r="E141" s="2" t="s">
-        <v>169</v>
+        <v>6</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B142" s="2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C142" s="2" t="s">
         <v>83</v>
@@ -3070,12 +3057,12 @@
         <v>156</v>
       </c>
       <c r="E142" s="2" t="s">
-        <v>169</v>
+        <v>6</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B143" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C143" s="2" t="s">
         <v>83</v>
@@ -3089,7 +3076,7 @@
     </row>
     <row r="144" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B144" s="2" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C144" s="2" t="s">
         <v>83</v>
@@ -3103,7 +3090,7 @@
     </row>
     <row r="145" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B145" s="2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C145" s="2" t="s">
         <v>83</v>
@@ -3117,7 +3104,7 @@
     </row>
     <row r="146" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B146" s="2" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C146" s="2" t="s">
         <v>83</v>
@@ -3131,7 +3118,7 @@
     </row>
     <row r="147" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B147" s="2" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C147" s="2" t="s">
         <v>83</v>
@@ -3140,12 +3127,12 @@
         <v>156</v>
       </c>
       <c r="E147" s="2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B148" s="2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C148" s="2" t="s">
         <v>83</v>
@@ -3157,7 +3144,7 @@
     </row>
     <row r="149" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B149" s="2" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C149" s="2" t="s">
         <v>83</v>
@@ -3169,7 +3156,7 @@
     </row>
     <row r="150" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B150" s="2" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C150" s="2" t="s">
         <v>83</v>
@@ -3181,7 +3168,7 @@
     </row>
     <row r="151" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B151" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C151" s="2" t="s">
         <v>83</v>
@@ -3193,7 +3180,7 @@
     </row>
     <row r="152" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B152" s="2" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C152" s="2" t="s">
         <v>83</v>
@@ -3205,7 +3192,7 @@
     </row>
     <row r="153" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B153" s="2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C153" s="2" t="s">
         <v>83</v>
@@ -3217,7 +3204,7 @@
     </row>
     <row r="154" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B154" s="2" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C154" s="2" t="s">
         <v>83</v>
@@ -3229,55 +3216,55 @@
     </row>
     <row r="155" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B155" s="2" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C155" s="2" t="s">
         <v>83</v>
       </c>
       <c r="D155" s="2"/>
-      <c r="E155" s="5" t="s">
-        <v>169</v>
+      <c r="E155" s="2" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B156" s="2" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C156" s="2" t="s">
         <v>83</v>
       </c>
       <c r="D156" s="2"/>
-      <c r="E156" s="5" t="s">
-        <v>169</v>
+      <c r="E156" s="2" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="157" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B157" s="2" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C157" s="2" t="s">
         <v>83</v>
       </c>
       <c r="D157" s="2"/>
-      <c r="E157" s="5" t="s">
-        <v>169</v>
+      <c r="E157" s="2" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="158" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B158" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="C158" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="C158" s="2" t="s">
         <v>83</v>
       </c>
       <c r="D158" s="2"/>
       <c r="E158" s="2" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="159" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B159" s="2" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C159" s="2" t="s">
         <v>83</v>
@@ -3289,13 +3276,13 @@
     </row>
     <row r="160" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B160" s="2" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C160" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="D160" s="2" t="s">
         <v>193</v>
-      </c>
-      <c r="D160" s="2" t="s">
-        <v>194</v>
       </c>
       <c r="E160" s="2" t="s">
         <v>67</v>
@@ -3303,13 +3290,13 @@
     </row>
     <row r="161" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B161" s="2" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C161" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="D161" s="2" t="s">
         <v>193</v>
-      </c>
-      <c r="D161" s="2" t="s">
-        <v>194</v>
       </c>
       <c r="E161" s="2" t="s">
         <v>67</v>
@@ -3317,13 +3304,13 @@
     </row>
     <row r="162" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B162" s="2" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C162" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="D162" s="2" t="s">
         <v>193</v>
-      </c>
-      <c r="D162" s="2" t="s">
-        <v>194</v>
       </c>
       <c r="E162" s="2" t="s">
         <v>67</v>
@@ -3331,13 +3318,13 @@
     </row>
     <row r="163" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B163" s="2" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C163" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="D163" s="2" t="s">
         <v>193</v>
-      </c>
-      <c r="D163" s="2" t="s">
-        <v>194</v>
       </c>
       <c r="E163" s="2" t="s">
         <v>63</v>
@@ -3345,13 +3332,13 @@
     </row>
     <row r="164" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B164" s="2" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C164" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="D164" s="2" t="s">
         <v>193</v>
-      </c>
-      <c r="D164" s="2" t="s">
-        <v>194</v>
       </c>
       <c r="E164" s="2" t="s">
         <v>63</v>
@@ -3359,13 +3346,13 @@
     </row>
     <row r="165" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B165" s="2" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C165" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="D165" s="2" t="s">
         <v>193</v>
-      </c>
-      <c r="D165" s="2" t="s">
-        <v>194</v>
       </c>
       <c r="E165" s="2" t="s">
         <v>63</v>
@@ -3373,13 +3360,13 @@
     </row>
     <row r="166" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B166" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="C166" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="D166" s="2" t="s">
         <v>200</v>
-      </c>
-      <c r="C166" s="2" t="s">
-        <v>193</v>
-      </c>
-      <c r="D166" s="2" t="s">
-        <v>201</v>
       </c>
       <c r="E166" s="2" t="s">
         <v>6</v>
@@ -3387,13 +3374,13 @@
     </row>
     <row r="167" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B167" s="2" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C167" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D167" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E167" s="2" t="s">
         <v>6</v>
@@ -3401,13 +3388,13 @@
     </row>
     <row r="168" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B168" s="2" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C168" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D168" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E168" s="2" t="s">
         <v>6</v>
@@ -3415,13 +3402,13 @@
     </row>
     <row r="169" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B169" s="2" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C169" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D169" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E169" s="2" t="s">
         <v>11</v>
@@ -3429,13 +3416,13 @@
     </row>
     <row r="170" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B170" s="2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C170" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D170" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E170" s="2" t="s">
         <v>11</v>
@@ -3443,13 +3430,13 @@
     </row>
     <row r="171" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B171" s="2" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C171" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D171" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E171" s="2" t="s">
         <v>11</v>
@@ -3457,13 +3444,13 @@
     </row>
     <row r="172" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B172" s="2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C172" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D172" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E172" s="2" t="s">
         <v>15</v>
@@ -3471,13 +3458,13 @@
     </row>
     <row r="173" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B173" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C173" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D173" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E173" s="2" t="s">
         <v>15</v>
@@ -3485,13 +3472,13 @@
     </row>
     <row r="174" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B174" s="2" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C174" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D174" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E174" s="2" t="s">
         <v>15</v>
@@ -3499,13 +3486,13 @@
     </row>
     <row r="175" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B175" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C175" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D175" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E175" s="2" t="s">
         <v>19</v>
@@ -3513,13 +3500,13 @@
     </row>
     <row r="176" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B176" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C176" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D176" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E176" s="2" t="s">
         <v>19</v>
@@ -3527,13 +3514,13 @@
     </row>
     <row r="177" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B177" s="2" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C177" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D177" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E177" s="2" t="s">
         <v>19</v>
@@ -3541,13 +3528,13 @@
     </row>
     <row r="178" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B178" s="2" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C178" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D178" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E178" s="2" t="s">
         <v>23</v>
@@ -3555,13 +3542,13 @@
     </row>
     <row r="179" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B179" s="2" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C179" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D179" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E179" s="2" t="s">
         <v>23</v>
@@ -3569,13 +3556,13 @@
     </row>
     <row r="180" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B180" s="2" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C180" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D180" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E180" s="2" t="s">
         <v>23</v>
@@ -3583,13 +3570,13 @@
     </row>
     <row r="181" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B181" s="2" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C181" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D181" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E181" s="2" t="s">
         <v>27</v>
@@ -3597,13 +3584,13 @@
     </row>
     <row r="182" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B182" s="2" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C182" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D182" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E182" s="2" t="s">
         <v>27</v>
@@ -3611,13 +3598,13 @@
     </row>
     <row r="183" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B183" s="2" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C183" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D183" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E183" s="2" t="s">
         <v>27</v>
@@ -3625,13 +3612,13 @@
     </row>
     <row r="184" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B184" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C184" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D184" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E184" s="2" t="s">
         <v>31</v>
@@ -3639,13 +3626,13 @@
     </row>
     <row r="185" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B185" s="2" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C185" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D185" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E185" s="2" t="s">
         <v>31</v>
@@ -3653,13 +3640,13 @@
     </row>
     <row r="186" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B186" s="2" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C186" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D186" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E186" s="2" t="s">
         <v>31</v>
@@ -3668,13 +3655,13 @@
     <row r="187" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A187" s="2"/>
       <c r="B187" s="4" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C187" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D187" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E187" s="2" t="s">
         <v>31</v>
@@ -3699,13 +3686,13 @@
     </row>
     <row r="188" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B188" s="2" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C188" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D188" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E188" s="2" t="s">
         <v>35</v>
@@ -3713,13 +3700,13 @@
     </row>
     <row r="189" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B189" s="2" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C189" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D189" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E189" s="2" t="s">
         <v>35</v>
@@ -3727,13 +3714,13 @@
     </row>
     <row r="190" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B190" s="2" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C190" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D190" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E190" s="2" t="s">
         <v>35</v>
@@ -3741,13 +3728,13 @@
     </row>
     <row r="191" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B191" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C191" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D191" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E191" s="2" t="s">
         <v>63</v>
@@ -3755,13 +3742,13 @@
     </row>
     <row r="192" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B192" s="2" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C192" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D192" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E192" s="2" t="s">
         <v>63</v>
@@ -3769,13 +3756,13 @@
     </row>
     <row r="193" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B193" s="2" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C193" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D193" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E193" s="2" t="s">
         <v>63</v>
@@ -3783,13 +3770,13 @@
     </row>
     <row r="194" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B194" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="C194" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="D194" s="2" t="s">
         <v>229</v>
-      </c>
-      <c r="C194" s="2" t="s">
-        <v>193</v>
-      </c>
-      <c r="D194" s="2" t="s">
-        <v>230</v>
       </c>
       <c r="E194" s="2" t="s">
         <v>39</v>
@@ -3797,13 +3784,13 @@
     </row>
     <row r="195" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B195" s="2" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C195" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D195" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E195" s="2" t="s">
         <v>39</v>
@@ -3811,13 +3798,13 @@
     </row>
     <row r="196" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B196" s="2" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C196" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D196" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E196" s="2" t="s">
         <v>39</v>
@@ -3825,13 +3812,13 @@
     </row>
     <row r="197" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B197" s="2" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C197" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D197" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E197" s="2" t="s">
         <v>43</v>
@@ -3839,13 +3826,13 @@
     </row>
     <row r="198" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B198" s="2" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C198" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D198" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E198" s="2" t="s">
         <v>43</v>
@@ -3853,13 +3840,13 @@
     </row>
     <row r="199" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B199" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C199" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D199" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E199" s="2" t="s">
         <v>43</v>
@@ -3867,13 +3854,13 @@
     </row>
     <row r="200" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B200" s="2" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C200" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D200" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E200" s="2" t="s">
         <v>47</v>
@@ -3881,13 +3868,13 @@
     </row>
     <row r="201" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B201" s="2" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C201" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D201" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E201" s="2" t="s">
         <v>47</v>
@@ -3895,13 +3882,13 @@
     </row>
     <row r="202" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B202" s="2" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C202" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D202" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E202" s="2" t="s">
         <v>47</v>
@@ -3909,13 +3896,13 @@
     </row>
     <row r="203" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B203" s="2" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C203" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D203" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E203" s="2" t="s">
         <v>51</v>
@@ -3923,13 +3910,13 @@
     </row>
     <row r="204" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B204" s="2" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C204" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D204" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E204" s="2" t="s">
         <v>51</v>
@@ -3937,13 +3924,13 @@
     </row>
     <row r="205" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B205" s="2" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C205" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D205" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E205" s="2" t="s">
         <v>51</v>
@@ -3951,13 +3938,13 @@
     </row>
     <row r="206" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B206" s="2" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C206" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D206" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E206" s="2" t="s">
         <v>55</v>
@@ -3965,13 +3952,13 @@
     </row>
     <row r="207" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B207" s="2" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C207" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D207" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E207" s="2" t="s">
         <v>55</v>
@@ -3979,13 +3966,13 @@
     </row>
     <row r="208" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B208" s="2" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C208" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D208" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E208" s="2" t="s">
         <v>55</v>
@@ -3993,13 +3980,13 @@
     </row>
     <row r="209" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B209" s="2" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C209" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D209" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E209" s="2" t="s">
         <v>59</v>
@@ -4007,13 +3994,13 @@
     </row>
     <row r="210" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B210" s="2" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C210" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D210" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E210" s="2" t="s">
         <v>59</v>
@@ -4021,13 +4008,13 @@
     </row>
     <row r="211" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B211" s="2" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C211" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D211" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E211" s="2" t="s">
         <v>59</v>
@@ -4035,13 +4022,13 @@
     </row>
     <row r="212" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B212" s="2" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C212" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D212" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E212" s="2" t="s">
         <v>81</v>
@@ -4049,7 +4036,7 @@
     </row>
     <row r="213" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B213" s="2" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C213" s="2" t="s">
         <v>5</v>
@@ -4063,7 +4050,7 @@
     </row>
     <row r="214" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B214" s="2" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C214" s="2" t="s">
         <v>5</v>
@@ -4077,7 +4064,7 @@
     </row>
     <row r="215" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B215" s="2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="C215" s="2" t="s">
         <v>5</v>
@@ -4091,13 +4078,13 @@
     </row>
     <row r="216" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B216" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="C216" s="5" t="s">
         <v>252</v>
       </c>
-      <c r="C216" s="6" t="s">
-        <v>253</v>
-      </c>
-      <c r="D216" s="6"/>
-      <c r="E216" s="6"/>
+      <c r="D216" s="5"/>
+      <c r="E216" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Changed XRF data to the newer version and rerun the analysis (Hausdorf)
</commit_message>
<xml_diff>
--- a/data/opis_uzupelniony.xlsx
+++ b/data/opis_uzupelniony.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="784" uniqueCount="253">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="824" uniqueCount="264">
   <si>
     <t xml:space="preserve">NAZWA</t>
   </si>
@@ -220,18 +220,30 @@
     <t xml:space="preserve">APP14C</t>
   </si>
   <si>
+    <t xml:space="preserve">APP14D</t>
+  </si>
+  <si>
     <t xml:space="preserve">APP15A</t>
   </si>
   <si>
     <t xml:space="preserve">poprawka </t>
   </si>
   <si>
+    <t xml:space="preserve">APP15A1</t>
+  </si>
+  <si>
     <t xml:space="preserve">APP15B</t>
   </si>
   <si>
+    <t xml:space="preserve">APP15B1</t>
+  </si>
+  <si>
     <t xml:space="preserve">APP15C</t>
   </si>
   <si>
+    <t xml:space="preserve">APP15C1</t>
+  </si>
+  <si>
     <t xml:space="preserve">APP15C2</t>
   </si>
   <si>
@@ -307,6 +319,9 @@
     <t xml:space="preserve">ASC2B</t>
   </si>
   <si>
+    <t xml:space="preserve">ASC2C</t>
+  </si>
+  <si>
     <t xml:space="preserve">ASC3</t>
   </si>
   <si>
@@ -346,6 +361,9 @@
     <t xml:space="preserve">ASC5B</t>
   </si>
   <si>
+    <t xml:space="preserve">ASC5C</t>
+  </si>
+  <si>
     <t xml:space="preserve">ASC6</t>
   </si>
   <si>
@@ -463,6 +481,9 @@
     <t xml:space="preserve">ASC14B</t>
   </si>
   <si>
+    <t xml:space="preserve">ASC14C</t>
+  </si>
+  <si>
     <t xml:space="preserve">ASC15</t>
   </si>
   <si>
@@ -499,6 +520,9 @@
     <t xml:space="preserve">ASC17B</t>
   </si>
   <si>
+    <t xml:space="preserve">ASC17C</t>
+  </si>
+  <si>
     <t xml:space="preserve">ASC18</t>
   </si>
   <si>
@@ -508,6 +532,9 @@
     <t xml:space="preserve">ASC18B</t>
   </si>
   <si>
+    <t xml:space="preserve">ASC18C</t>
+  </si>
+  <si>
     <t xml:space="preserve">ASC19</t>
   </si>
   <si>
@@ -517,6 +544,9 @@
     <t xml:space="preserve">ASC19A2</t>
   </si>
   <si>
+    <t xml:space="preserve">ASC19B</t>
+  </si>
+  <si>
     <t xml:space="preserve">ASC19B1</t>
   </si>
   <si>
@@ -548,6 +578,9 @@
   </si>
   <si>
     <t xml:space="preserve">ASC21C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASC21D</t>
   </si>
   <si>
     <t xml:space="preserve">ASC22</t>
@@ -1082,7 +1115,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:V216"/>
+  <dimension ref="A1:V227"/>
   <sheetFormatPr defaultColWidth="12.66796875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5.78"/>
@@ -1757,22 +1790,22 @@
       </c>
     </row>
     <row r="49" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B49" s="3" t="s">
+      <c r="B49" s="2" t="s">
         <v>66</v>
       </c>
       <c r="C49" s="2" t="s">
         <v>5</v>
       </c>
       <c r="D49" s="2" t="n">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B50" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C50" s="2" t="s">
         <v>5</v>
@@ -1781,7 +1814,7 @@
         <v>77</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1795,11 +1828,11 @@
         <v>77</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B52" s="4" t="s">
+      <c r="B52" s="3" t="s">
         <v>70</v>
       </c>
       <c r="C52" s="2" t="s">
@@ -1809,11 +1842,11 @@
         <v>77</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B53" s="4" t="s">
+      <c r="B53" s="3" t="s">
         <v>71</v>
       </c>
       <c r="C53" s="2" t="s">
@@ -1823,11 +1856,11 @@
         <v>77</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B54" s="4" t="s">
+      <c r="B54" s="3" t="s">
         <v>72</v>
       </c>
       <c r="C54" s="2" t="s">
@@ -1837,67 +1870,75 @@
         <v>77</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B55" s="4" t="s">
+      <c r="B55" s="3" t="s">
         <v>73</v>
       </c>
       <c r="C55" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D55" s="2"/>
+      <c r="D55" s="2" t="n">
+        <v>77</v>
+      </c>
       <c r="E55" s="2" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B56" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C56" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D56" s="2"/>
+      <c r="D56" s="2" t="n">
+        <v>77</v>
+      </c>
       <c r="E56" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B57" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C57" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D57" s="2"/>
+      <c r="D57" s="2" t="n">
+        <v>77</v>
+      </c>
       <c r="E57" s="2" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B58" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D58" s="2" t="n">
         <v>77</v>
       </c>
-      <c r="C58" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D58" s="2"/>
       <c r="E58" s="2" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B59" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C59" s="2" t="s">
         <v>5</v>
       </c>
       <c r="D59" s="2"/>
       <c r="E59" s="2" t="s">
-        <v>63</v>
+        <v>78</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1909,91 +1950,83 @@
       </c>
       <c r="D60" s="2"/>
       <c r="E60" s="2" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B61" s="2" t="s">
+      <c r="B61" s="4" t="s">
         <v>80</v>
       </c>
       <c r="C61" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D61" s="2" t="n">
-        <v>84</v>
-      </c>
+      <c r="D61" s="2"/>
       <c r="E61" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B62" s="4" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="62" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B62" s="2" t="s">
+      <c r="C62" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D62" s="2"/>
+      <c r="E62" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B63" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="C62" s="2" t="s">
+      <c r="C63" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D63" s="2"/>
+      <c r="E63" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B64" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="D62" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="E62" s="2" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="63" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B63" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="C63" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="D63" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="E63" s="2" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="64" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B64" s="2" t="s">
-        <v>86</v>
-      </c>
       <c r="C64" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="D64" s="2" t="s">
-        <v>84</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="D64" s="2"/>
       <c r="E64" s="2" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B65" s="2" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="D65" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D65" s="2" t="n">
         <v>84</v>
       </c>
       <c r="E65" s="2" t="s">
-        <v>74</v>
+        <v>85</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B66" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="D66" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="C66" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="D66" s="2" t="s">
-        <v>84</v>
-      </c>
       <c r="E66" s="2" t="s">
-        <v>63</v>
+        <v>78</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2001,13 +2034,13 @@
         <v>89</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>63</v>
+        <v>78</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2015,13 +2048,13 @@
         <v>90</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="E68" s="2" t="s">
-        <v>63</v>
+        <v>78</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2029,13 +2062,13 @@
         <v>91</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>63</v>
+        <v>78</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2043,13 +2076,13 @@
         <v>92</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2057,13 +2090,13 @@
         <v>93</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="E71" s="2" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2071,13 +2104,13 @@
         <v>94</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2085,83 +2118,83 @@
         <v>95</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="E73" s="2" t="s">
-        <v>96</v>
+        <v>63</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B74" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="E74" s="2" t="s">
-        <v>96</v>
+        <v>68</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B75" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="E75" s="2" t="s">
-        <v>96</v>
+        <v>68</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B76" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="E76" s="2" t="s">
-        <v>96</v>
+        <v>68</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B77" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="E77" s="2" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B78" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="C78" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="D78" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="E78" s="2" t="s">
         <v>101</v>
-      </c>
-      <c r="C78" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="D78" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="E78" s="2" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2169,13 +2202,13 @@
         <v>102</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="E79" s="2" t="s">
-        <v>63</v>
+        <v>101</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2183,13 +2216,13 @@
         <v>103</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="E80" s="2" t="s">
-        <v>63</v>
+        <v>101</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2197,52 +2230,52 @@
         <v>104</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>105</v>
+        <v>88</v>
       </c>
       <c r="E81" s="2" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B82" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>105</v>
+        <v>88</v>
       </c>
       <c r="E82" s="2" t="s">
-        <v>96</v>
+        <v>63</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B83" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>105</v>
+        <v>88</v>
       </c>
       <c r="E83" s="2" t="s">
-        <v>96</v>
+        <v>63</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B84" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>105</v>
+        <v>88</v>
       </c>
       <c r="E84" s="2" t="s">
         <v>63</v>
@@ -2250,13 +2283,13 @@
     </row>
     <row r="85" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B85" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>105</v>
+        <v>88</v>
       </c>
       <c r="E85" s="2" t="s">
         <v>63</v>
@@ -2264,16 +2297,16 @@
     </row>
     <row r="86" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B86" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C86" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="D86" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="C86" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="D86" s="2" t="s">
-        <v>105</v>
-      </c>
       <c r="E86" s="2" t="s">
-        <v>63</v>
+        <v>101</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2281,13 +2314,13 @@
         <v>111</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="E87" s="2" t="s">
-        <v>63</v>
+        <v>101</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2295,66 +2328,66 @@
         <v>112</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="E88" s="2" t="s">
-        <v>67</v>
+        <v>101</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B89" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="E89" s="2" t="s">
-        <v>67</v>
+        <v>101</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B90" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="E90" s="2" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B91" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="E91" s="2" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B92" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="E92" s="2" t="s">
         <v>63</v>
@@ -2362,13 +2395,13 @@
     </row>
     <row r="93" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B93" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="E93" s="2" t="s">
         <v>63</v>
@@ -2376,16 +2409,16 @@
     </row>
     <row r="94" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B94" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="C94" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="D94" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="C94" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="D94" s="2" t="s">
-        <v>113</v>
-      </c>
       <c r="E94" s="2" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2393,13 +2426,13 @@
         <v>120</v>
       </c>
       <c r="C95" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D95" s="2" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="E95" s="2" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2407,66 +2440,66 @@
         <v>121</v>
       </c>
       <c r="C96" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E96" s="2" t="s">
-        <v>96</v>
+        <v>68</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B97" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C97" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E97" s="2" t="s">
-        <v>96</v>
+        <v>68</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B98" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C98" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E98" s="2" t="s">
-        <v>96</v>
+        <v>63</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B99" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C99" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D99" s="2" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E99" s="2" t="s">
-        <v>96</v>
+        <v>63</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B100" s="2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C100" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D100" s="2" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E100" s="2" t="s">
         <v>63</v>
@@ -2474,13 +2507,13 @@
     </row>
     <row r="101" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B101" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C101" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D101" s="2" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E101" s="2" t="s">
         <v>63</v>
@@ -2488,16 +2521,16 @@
     </row>
     <row r="102" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B102" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C102" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="D102" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="C102" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="D102" s="2" t="s">
-        <v>122</v>
-      </c>
       <c r="E102" s="2" t="s">
-        <v>63</v>
+        <v>101</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2505,13 +2538,13 @@
         <v>129</v>
       </c>
       <c r="C103" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D103" s="2" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="E103" s="2" t="s">
-        <v>63</v>
+        <v>101</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2519,66 +2552,66 @@
         <v>130</v>
       </c>
       <c r="C104" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D104" s="2" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="E104" s="2" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B105" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C105" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D105" s="2" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="E105" s="2" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B106" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C106" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D106" s="2" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="E106" s="2" t="s">
-        <v>96</v>
+        <v>63</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B107" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C107" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D107" s="2" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="E107" s="2" t="s">
-        <v>96</v>
+        <v>63</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B108" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C108" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D108" s="2" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="E108" s="2" t="s">
         <v>63</v>
@@ -2586,13 +2619,13 @@
     </row>
     <row r="109" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B109" s="2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C109" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D109" s="2" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="E109" s="2" t="s">
         <v>63</v>
@@ -2600,16 +2633,16 @@
     </row>
     <row r="110" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B110" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="C110" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="D110" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="C110" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="D110" s="2" t="s">
-        <v>131</v>
-      </c>
       <c r="E110" s="2" t="s">
-        <v>63</v>
+        <v>101</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2617,13 +2650,13 @@
         <v>138</v>
       </c>
       <c r="C111" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D111" s="2" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="E111" s="2" t="s">
-        <v>63</v>
+        <v>101</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2631,13 +2664,13 @@
         <v>139</v>
       </c>
       <c r="C112" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D112" s="2" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="E112" s="2" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2645,13 +2678,13 @@
         <v>140</v>
       </c>
       <c r="C113" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D113" s="2" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="E113" s="2" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2659,13 +2692,13 @@
         <v>141</v>
       </c>
       <c r="C114" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D114" s="2" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="E114" s="2" t="s">
-        <v>96</v>
+        <v>63</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2673,13 +2706,13 @@
         <v>142</v>
       </c>
       <c r="C115" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D115" s="2" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="E115" s="2" t="s">
-        <v>96</v>
+        <v>63</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2687,97 +2720,97 @@
         <v>143</v>
       </c>
       <c r="C116" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D116" s="2" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="E116" s="2" t="s">
-        <v>96</v>
+        <v>63</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B117" s="2" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C117" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D117" s="2" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="E117" s="2" t="s">
-        <v>96</v>
+        <v>63</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B118" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C118" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D118" s="2" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="E118" s="2" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B119" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C119" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D119" s="2" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="E119" s="2" t="s">
-        <v>67</v>
+        <v>101</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B120" s="2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C120" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D120" s="2" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="E120" s="2" t="s">
-        <v>67</v>
+        <v>101</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B121" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C121" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D121" s="2" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="E121" s="2" t="s">
-        <v>67</v>
+        <v>101</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B122" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="C122" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="D122" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="C122" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="D122" s="2" t="s">
-        <v>144</v>
-      </c>
       <c r="E122" s="2" t="s">
-        <v>67</v>
+        <v>101</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2785,13 +2818,13 @@
         <v>151</v>
       </c>
       <c r="C123" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D123" s="2" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="E123" s="2" t="s">
-        <v>63</v>
+        <v>101</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2799,13 +2832,13 @@
         <v>152</v>
       </c>
       <c r="C124" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D124" s="2" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="E124" s="2" t="s">
-        <v>63</v>
+        <v>101</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2813,13 +2846,13 @@
         <v>153</v>
       </c>
       <c r="C125" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D125" s="2" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="E125" s="2" t="s">
-        <v>63</v>
+        <v>101</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2827,13 +2860,13 @@
         <v>154</v>
       </c>
       <c r="C126" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D126" s="2" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="E126" s="2" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2841,94 +2874,94 @@
         <v>155</v>
       </c>
       <c r="C127" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D127" s="2" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="E127" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B128" s="2" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C128" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D128" s="2" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="E128" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B129" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C129" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D129" s="2" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="E129" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B130" s="2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C130" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D130" s="2" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="E130" s="2" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B131" s="2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C131" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D131" s="2" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="E131" s="2" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B132" s="2" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C132" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D132" s="2" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="E132" s="2" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B133" s="2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C133" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D133" s="2" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="E133" s="2" t="s">
         <v>63</v>
@@ -2936,16 +2969,16 @@
     </row>
     <row r="134" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B134" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="C134" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="D134" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="C134" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="D134" s="2" t="s">
-        <v>156</v>
-      </c>
       <c r="E134" s="2" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2953,13 +2986,13 @@
         <v>164</v>
       </c>
       <c r="C135" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D135" s="2" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="E135" s="2" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2967,13 +3000,13 @@
         <v>165</v>
       </c>
       <c r="C136" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D136" s="2" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="E136" s="2" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2981,13 +3014,13 @@
         <v>166</v>
       </c>
       <c r="C137" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D137" s="2" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="E137" s="2" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2995,13 +3028,13 @@
         <v>167</v>
       </c>
       <c r="C138" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D138" s="2" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="E138" s="2" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3009,13 +3042,13 @@
         <v>168</v>
       </c>
       <c r="C139" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D139" s="2" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="E139" s="2" t="s">
-        <v>6</v>
+        <v>68</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3023,13 +3056,13 @@
         <v>169</v>
       </c>
       <c r="C140" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D140" s="2" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="E140" s="2" t="s">
-        <v>6</v>
+        <v>68</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3037,13 +3070,13 @@
         <v>170</v>
       </c>
       <c r="C141" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D141" s="2" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="E141" s="2" t="s">
-        <v>6</v>
+        <v>68</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3051,13 +3084,13 @@
         <v>171</v>
       </c>
       <c r="C142" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D142" s="2" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="E142" s="2" t="s">
-        <v>6</v>
+        <v>63</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3065,13 +3098,13 @@
         <v>172</v>
       </c>
       <c r="C143" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D143" s="2" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="E143" s="2" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3079,13 +3112,13 @@
         <v>173</v>
       </c>
       <c r="C144" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D144" s="2" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="E144" s="2" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3093,13 +3126,13 @@
         <v>174</v>
       </c>
       <c r="C145" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D145" s="2" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="E145" s="2" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3107,13 +3140,13 @@
         <v>175</v>
       </c>
       <c r="C146" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D146" s="2" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="E146" s="2" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3121,409 +3154,409 @@
         <v>176</v>
       </c>
       <c r="C147" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D147" s="2" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="E147" s="2" t="s">
-        <v>177</v>
+        <v>63</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B148" s="2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C148" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="D148" s="2"/>
+        <v>87</v>
+      </c>
+      <c r="D148" s="2" t="s">
+        <v>163</v>
+      </c>
       <c r="E148" s="2" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B149" s="2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C149" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="D149" s="2"/>
+        <v>87</v>
+      </c>
+      <c r="D149" s="2" t="s">
+        <v>163</v>
+      </c>
       <c r="E149" s="2" t="s">
-        <v>67</v>
+        <v>6</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B150" s="2" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C150" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="D150" s="2"/>
+        <v>87</v>
+      </c>
+      <c r="D150" s="2" t="s">
+        <v>163</v>
+      </c>
       <c r="E150" s="2" t="s">
-        <v>67</v>
+        <v>6</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B151" s="2" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C151" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="D151" s="2"/>
+        <v>87</v>
+      </c>
+      <c r="D151" s="2" t="s">
+        <v>163</v>
+      </c>
       <c r="E151" s="2" t="s">
-        <v>67</v>
+        <v>6</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B152" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C152" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="D152" s="2"/>
+        <v>87</v>
+      </c>
+      <c r="D152" s="2" t="s">
+        <v>163</v>
+      </c>
       <c r="E152" s="2" t="s">
-        <v>63</v>
+        <v>6</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B153" s="2" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C153" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="D153" s="2"/>
+        <v>87</v>
+      </c>
+      <c r="D153" s="2" t="s">
+        <v>163</v>
+      </c>
       <c r="E153" s="2" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B154" s="2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C154" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="D154" s="2"/>
+        <v>87</v>
+      </c>
+      <c r="D154" s="2" t="s">
+        <v>163</v>
+      </c>
       <c r="E154" s="2" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B155" s="2" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C155" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="D155" s="2"/>
+        <v>87</v>
+      </c>
+      <c r="D155" s="2" t="s">
+        <v>163</v>
+      </c>
       <c r="E155" s="2" t="s">
-        <v>6</v>
+        <v>59</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B156" s="2" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C156" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="D156" s="2"/>
+        <v>87</v>
+      </c>
+      <c r="D156" s="2" t="s">
+        <v>163</v>
+      </c>
       <c r="E156" s="2" t="s">
-        <v>6</v>
+        <v>59</v>
       </c>
     </row>
     <row r="157" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B157" s="2" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C157" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="D157" s="2"/>
+        <v>87</v>
+      </c>
+      <c r="D157" s="2" t="s">
+        <v>163</v>
+      </c>
       <c r="E157" s="2" t="s">
-        <v>6</v>
+        <v>59</v>
       </c>
     </row>
     <row r="158" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B158" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="C158" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="D158" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="E158" s="2" t="s">
         <v>188</v>
-      </c>
-      <c r="C158" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="D158" s="2"/>
-      <c r="E158" s="2" t="s">
-        <v>189</v>
       </c>
     </row>
     <row r="159" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B159" s="2" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C159" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D159" s="2"/>
       <c r="E159" s="2" t="s">
-        <v>81</v>
+        <v>68</v>
       </c>
     </row>
     <row r="160" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B160" s="2" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C160" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="D160" s="2" t="s">
-        <v>193</v>
-      </c>
+        <v>87</v>
+      </c>
+      <c r="D160" s="2"/>
       <c r="E160" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="161" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B161" s="2" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="C161" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="D161" s="2" t="s">
-        <v>193</v>
-      </c>
+        <v>87</v>
+      </c>
+      <c r="D161" s="2"/>
       <c r="E161" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="162" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B162" s="2" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="C162" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="D162" s="2" t="s">
-        <v>193</v>
-      </c>
+        <v>87</v>
+      </c>
+      <c r="D162" s="2"/>
       <c r="E162" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="163" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B163" s="2" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="C163" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="D163" s="2" t="s">
-        <v>193</v>
-      </c>
+        <v>87</v>
+      </c>
+      <c r="D163" s="2"/>
       <c r="E163" s="2" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="164" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B164" s="2" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="C164" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="D164" s="2" t="s">
-        <v>193</v>
-      </c>
+        <v>87</v>
+      </c>
+      <c r="D164" s="2"/>
       <c r="E164" s="2" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="165" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B165" s="2" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="C165" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="D165" s="2" t="s">
-        <v>193</v>
-      </c>
+        <v>87</v>
+      </c>
+      <c r="D165" s="2"/>
       <c r="E165" s="2" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="166" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B166" s="2" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="C166" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="D166" s="2" t="s">
-        <v>200</v>
-      </c>
+        <v>87</v>
+      </c>
+      <c r="D166" s="2"/>
       <c r="E166" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="167" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B167" s="2" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="C167" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="D167" s="2" t="s">
-        <v>200</v>
-      </c>
+        <v>87</v>
+      </c>
+      <c r="D167" s="2"/>
       <c r="E167" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="168" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B168" s="2" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="C168" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="D168" s="2" t="s">
-        <v>200</v>
-      </c>
+        <v>87</v>
+      </c>
+      <c r="D168" s="2"/>
       <c r="E168" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="169" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B169" s="2" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="C169" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="D169" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="D169" s="2"/>
+      <c r="E169" s="2" t="s">
         <v>200</v>
-      </c>
-      <c r="E169" s="2" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="170" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B170" s="2" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="C170" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="D170" s="2" t="s">
-        <v>200</v>
-      </c>
+        <v>87</v>
+      </c>
+      <c r="D170" s="2"/>
       <c r="E170" s="2" t="s">
-        <v>11</v>
+        <v>85</v>
       </c>
     </row>
     <row r="171" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B171" s="2" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="C171" s="2" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="D171" s="2" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="E171" s="2" t="s">
-        <v>11</v>
+        <v>68</v>
       </c>
     </row>
     <row r="172" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B172" s="2" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C172" s="2" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="D172" s="2" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="E172" s="2" t="s">
-        <v>15</v>
+        <v>68</v>
       </c>
     </row>
     <row r="173" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B173" s="2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C173" s="2" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="D173" s="2" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="E173" s="2" t="s">
-        <v>15</v>
+        <v>68</v>
       </c>
     </row>
     <row r="174" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B174" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C174" s="2" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="D174" s="2" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="E174" s="2" t="s">
-        <v>15</v>
+        <v>63</v>
       </c>
     </row>
     <row r="175" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B175" s="2" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C175" s="2" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="D175" s="2" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="E175" s="2" t="s">
-        <v>19</v>
+        <v>63</v>
       </c>
     </row>
     <row r="176" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B176" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C176" s="2" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="D176" s="2" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="E176" s="2" t="s">
-        <v>19</v>
+        <v>63</v>
       </c>
     </row>
     <row r="177" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B177" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="C177" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="D177" s="2" t="s">
         <v>211</v>
       </c>
-      <c r="C177" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="D177" s="2" t="s">
-        <v>200</v>
-      </c>
       <c r="E177" s="2" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
     </row>
     <row r="178" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3531,13 +3564,13 @@
         <v>212</v>
       </c>
       <c r="C178" s="2" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="D178" s="2" t="s">
-        <v>200</v>
+        <v>211</v>
       </c>
       <c r="E178" s="2" t="s">
-        <v>23</v>
+        <v>6</v>
       </c>
     </row>
     <row r="179" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3545,13 +3578,13 @@
         <v>213</v>
       </c>
       <c r="C179" s="2" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="D179" s="2" t="s">
-        <v>200</v>
+        <v>211</v>
       </c>
       <c r="E179" s="2" t="s">
-        <v>23</v>
+        <v>6</v>
       </c>
     </row>
     <row r="180" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3559,13 +3592,13 @@
         <v>214</v>
       </c>
       <c r="C180" s="2" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="D180" s="2" t="s">
-        <v>200</v>
+        <v>211</v>
       </c>
       <c r="E180" s="2" t="s">
-        <v>23</v>
+        <v>11</v>
       </c>
     </row>
     <row r="181" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3573,13 +3606,13 @@
         <v>215</v>
       </c>
       <c r="C181" s="2" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="D181" s="2" t="s">
-        <v>200</v>
+        <v>211</v>
       </c>
       <c r="E181" s="2" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
     </row>
     <row r="182" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3587,13 +3620,13 @@
         <v>216</v>
       </c>
       <c r="C182" s="2" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="D182" s="2" t="s">
-        <v>200</v>
+        <v>211</v>
       </c>
       <c r="E182" s="2" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
     </row>
     <row r="183" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3601,27 +3634,27 @@
         <v>217</v>
       </c>
       <c r="C183" s="2" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="D183" s="2" t="s">
-        <v>200</v>
+        <v>211</v>
       </c>
       <c r="E183" s="2" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
     </row>
     <row r="184" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B184" s="3" t="s">
+      <c r="B184" s="2" t="s">
         <v>218</v>
       </c>
       <c r="C184" s="2" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="D184" s="2" t="s">
-        <v>200</v>
+        <v>211</v>
       </c>
       <c r="E184" s="2" t="s">
-        <v>31</v>
+        <v>15</v>
       </c>
     </row>
     <row r="185" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3629,13 +3662,13 @@
         <v>219</v>
       </c>
       <c r="C185" s="2" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="D185" s="2" t="s">
-        <v>200</v>
+        <v>211</v>
       </c>
       <c r="E185" s="2" t="s">
-        <v>31</v>
+        <v>15</v>
       </c>
     </row>
     <row r="186" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3643,59 +3676,41 @@
         <v>220</v>
       </c>
       <c r="C186" s="2" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="D186" s="2" t="s">
-        <v>200</v>
+        <v>211</v>
       </c>
       <c r="E186" s="2" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
     </row>
     <row r="187" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A187" s="2"/>
-      <c r="B187" s="4" t="s">
+      <c r="B187" s="2" t="s">
         <v>221</v>
       </c>
       <c r="C187" s="2" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="D187" s="2" t="s">
-        <v>200</v>
+        <v>211</v>
       </c>
       <c r="E187" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="F187" s="2"/>
-      <c r="G187" s="2"/>
-      <c r="H187" s="2"/>
-      <c r="I187" s="2"/>
-      <c r="J187" s="2"/>
-      <c r="K187" s="2"/>
-      <c r="L187" s="2"/>
-      <c r="M187" s="2"/>
-      <c r="N187" s="2"/>
-      <c r="O187" s="2"/>
-      <c r="P187" s="2"/>
-      <c r="Q187" s="2"/>
-      <c r="R187" s="2"/>
-      <c r="S187" s="2"/>
-      <c r="T187" s="2"/>
-      <c r="U187" s="2"/>
-      <c r="V187" s="2"/>
+        <v>19</v>
+      </c>
     </row>
     <row r="188" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B188" s="2" t="s">
         <v>222</v>
       </c>
       <c r="C188" s="2" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="D188" s="2" t="s">
-        <v>200</v>
+        <v>211</v>
       </c>
       <c r="E188" s="2" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
     </row>
     <row r="189" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3703,13 +3718,13 @@
         <v>223</v>
       </c>
       <c r="C189" s="2" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="D189" s="2" t="s">
-        <v>200</v>
+        <v>211</v>
       </c>
       <c r="E189" s="2" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
     </row>
     <row r="190" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3717,13 +3732,13 @@
         <v>224</v>
       </c>
       <c r="C190" s="2" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="D190" s="2" t="s">
-        <v>200</v>
+        <v>211</v>
       </c>
       <c r="E190" s="2" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
     </row>
     <row r="191" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3731,13 +3746,13 @@
         <v>225</v>
       </c>
       <c r="C191" s="2" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="D191" s="2" t="s">
-        <v>200</v>
+        <v>211</v>
       </c>
       <c r="E191" s="2" t="s">
-        <v>63</v>
+        <v>23</v>
       </c>
     </row>
     <row r="192" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3745,13 +3760,13 @@
         <v>226</v>
       </c>
       <c r="C192" s="2" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="D192" s="2" t="s">
-        <v>200</v>
+        <v>211</v>
       </c>
       <c r="E192" s="2" t="s">
-        <v>63</v>
+        <v>27</v>
       </c>
     </row>
     <row r="193" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3759,13 +3774,13 @@
         <v>227</v>
       </c>
       <c r="C193" s="2" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="D193" s="2" t="s">
-        <v>200</v>
+        <v>211</v>
       </c>
       <c r="E193" s="2" t="s">
-        <v>63</v>
+        <v>27</v>
       </c>
     </row>
     <row r="194" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3773,167 +3788,185 @@
         <v>228</v>
       </c>
       <c r="C194" s="2" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="D194" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="E194" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="195" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B195" s="3" t="s">
         <v>229</v>
       </c>
-      <c r="E194" s="2" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="195" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B195" s="2" t="s">
-        <v>230</v>
-      </c>
       <c r="C195" s="2" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="D195" s="2" t="s">
-        <v>229</v>
+        <v>211</v>
       </c>
       <c r="E195" s="2" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
     </row>
     <row r="196" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B196" s="2" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C196" s="2" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="D196" s="2" t="s">
-        <v>229</v>
+        <v>211</v>
       </c>
       <c r="E196" s="2" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
     </row>
     <row r="197" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B197" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="C197" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="D197" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="E197" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="198" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A198" s="2"/>
+      <c r="B198" s="4" t="s">
         <v>232</v>
       </c>
-      <c r="C197" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="D197" s="2" t="s">
-        <v>229</v>
-      </c>
-      <c r="E197" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="198" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B198" s="2" t="s">
-        <v>233</v>
-      </c>
       <c r="C198" s="2" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="D198" s="2" t="s">
-        <v>229</v>
+        <v>211</v>
       </c>
       <c r="E198" s="2" t="s">
-        <v>43</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="F198" s="2"/>
+      <c r="G198" s="2"/>
+      <c r="H198" s="2"/>
+      <c r="I198" s="2"/>
+      <c r="J198" s="2"/>
+      <c r="K198" s="2"/>
+      <c r="L198" s="2"/>
+      <c r="M198" s="2"/>
+      <c r="N198" s="2"/>
+      <c r="O198" s="2"/>
+      <c r="P198" s="2"/>
+      <c r="Q198" s="2"/>
+      <c r="R198" s="2"/>
+      <c r="S198" s="2"/>
+      <c r="T198" s="2"/>
+      <c r="U198" s="2"/>
+      <c r="V198" s="2"/>
     </row>
     <row r="199" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B199" s="2" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C199" s="2" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="D199" s="2" t="s">
-        <v>229</v>
+        <v>211</v>
       </c>
       <c r="E199" s="2" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
     </row>
     <row r="200" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B200" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C200" s="2" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="D200" s="2" t="s">
-        <v>229</v>
+        <v>211</v>
       </c>
       <c r="E200" s="2" t="s">
-        <v>47</v>
+        <v>35</v>
       </c>
     </row>
     <row r="201" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B201" s="2" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C201" s="2" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="D201" s="2" t="s">
-        <v>229</v>
+        <v>211</v>
       </c>
       <c r="E201" s="2" t="s">
-        <v>47</v>
+        <v>35</v>
       </c>
     </row>
     <row r="202" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B202" s="2" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C202" s="2" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="D202" s="2" t="s">
-        <v>229</v>
+        <v>211</v>
       </c>
       <c r="E202" s="2" t="s">
-        <v>47</v>
+        <v>63</v>
       </c>
     </row>
     <row r="203" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B203" s="2" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C203" s="2" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="D203" s="2" t="s">
-        <v>229</v>
+        <v>211</v>
       </c>
       <c r="E203" s="2" t="s">
-        <v>51</v>
+        <v>63</v>
       </c>
     </row>
     <row r="204" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B204" s="2" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C204" s="2" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="D204" s="2" t="s">
-        <v>229</v>
+        <v>211</v>
       </c>
       <c r="E204" s="2" t="s">
-        <v>51</v>
+        <v>63</v>
       </c>
     </row>
     <row r="205" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B205" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="C205" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="D205" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="C205" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="D205" s="2" t="s">
-        <v>229</v>
-      </c>
       <c r="E205" s="2" t="s">
-        <v>51</v>
+        <v>39</v>
       </c>
     </row>
     <row r="206" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3941,13 +3974,13 @@
         <v>241</v>
       </c>
       <c r="C206" s="2" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="D206" s="2" t="s">
-        <v>229</v>
+        <v>240</v>
       </c>
       <c r="E206" s="2" t="s">
-        <v>55</v>
+        <v>39</v>
       </c>
     </row>
     <row r="207" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3955,13 +3988,13 @@
         <v>242</v>
       </c>
       <c r="C207" s="2" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="D207" s="2" t="s">
-        <v>229</v>
+        <v>240</v>
       </c>
       <c r="E207" s="2" t="s">
-        <v>55</v>
+        <v>39</v>
       </c>
     </row>
     <row r="208" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3969,13 +4002,13 @@
         <v>243</v>
       </c>
       <c r="C208" s="2" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="D208" s="2" t="s">
-        <v>229</v>
+        <v>240</v>
       </c>
       <c r="E208" s="2" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
     </row>
     <row r="209" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3983,13 +4016,13 @@
         <v>244</v>
       </c>
       <c r="C209" s="2" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="D209" s="2" t="s">
-        <v>229</v>
+        <v>240</v>
       </c>
       <c r="E209" s="2" t="s">
-        <v>59</v>
+        <v>43</v>
       </c>
     </row>
     <row r="210" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3997,13 +4030,13 @@
         <v>245</v>
       </c>
       <c r="C210" s="2" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="D210" s="2" t="s">
-        <v>229</v>
+        <v>240</v>
       </c>
       <c r="E210" s="2" t="s">
-        <v>59</v>
+        <v>43</v>
       </c>
     </row>
     <row r="211" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4011,13 +4044,13 @@
         <v>246</v>
       </c>
       <c r="C211" s="2" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="D211" s="2" t="s">
-        <v>229</v>
+        <v>240</v>
       </c>
       <c r="E211" s="2" t="s">
-        <v>59</v>
+        <v>47</v>
       </c>
     </row>
     <row r="212" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4025,13 +4058,13 @@
         <v>247</v>
       </c>
       <c r="C212" s="2" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="D212" s="2" t="s">
-        <v>200</v>
+        <v>240</v>
       </c>
       <c r="E212" s="2" t="s">
-        <v>81</v>
+        <v>47</v>
       </c>
     </row>
     <row r="213" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4039,13 +4072,13 @@
         <v>248</v>
       </c>
       <c r="C213" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D213" s="2" t="n">
-        <v>74</v>
+        <v>203</v>
+      </c>
+      <c r="D213" s="2" t="s">
+        <v>240</v>
       </c>
       <c r="E213" s="2" t="s">
-        <v>74</v>
+        <v>47</v>
       </c>
     </row>
     <row r="214" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4053,13 +4086,13 @@
         <v>249</v>
       </c>
       <c r="C214" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D214" s="2" t="n">
-        <v>74</v>
+        <v>203</v>
+      </c>
+      <c r="D214" s="2" t="s">
+        <v>240</v>
       </c>
       <c r="E214" s="2" t="s">
-        <v>74</v>
+        <v>51</v>
       </c>
     </row>
     <row r="215" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4067,28 +4100,182 @@
         <v>250</v>
       </c>
       <c r="C215" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D215" s="2" t="n">
-        <v>74</v>
+        <v>203</v>
+      </c>
+      <c r="D215" s="2" t="s">
+        <v>240</v>
       </c>
       <c r="E215" s="2" t="s">
-        <v>74</v>
+        <v>51</v>
       </c>
     </row>
     <row r="216" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B216" s="2" t="s">
         <v>251</v>
       </c>
-      <c r="C216" s="5" t="s">
+      <c r="C216" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="D216" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="E216" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="217" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B217" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="D216" s="5"/>
-      <c r="E216" s="5"/>
+      <c r="C217" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="D217" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="E217" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="218" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B218" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="C218" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="D218" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="E218" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="219" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B219" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="C219" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="D219" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="E219" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="220" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B220" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="C220" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="D220" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="E220" s="2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="221" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B221" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="C221" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="D221" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="E221" s="2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="222" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B222" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="C222" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="D222" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="E222" s="2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="223" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B223" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="C223" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="D223" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="E223" s="2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="224" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B224" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="C224" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D224" s="2" t="n">
+        <v>74</v>
+      </c>
+      <c r="E224" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="225" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B225" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="C225" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D225" s="2" t="n">
+        <v>74</v>
+      </c>
+      <c r="E225" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="226" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B226" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="C226" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D226" s="2" t="n">
+        <v>74</v>
+      </c>
+      <c r="E226" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="227" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B227" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="C227" s="5" t="s">
+        <v>263</v>
+      </c>
+      <c r="D227" s="5"/>
+      <c r="E227" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="C216:E216"/>
+    <mergeCell ref="C227:E227"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>